<commit_message>
base run without exclusive rule
</commit_message>
<xml_diff>
--- a/dataset_agreed/saved_models/baserun/pointcloud_base_run1/epoch_10/per_file_predictions_epoch_10.xlsx
+++ b/dataset_agreed/saved_models/baserun/pointcloud_base_run1/epoch_10/per_file_predictions_epoch_10.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="521">
   <si>
     <t>Filename</t>
   </si>
@@ -808,769 +808,775 @@
     <t>0,1,1,0</t>
   </si>
   <si>
-    <t>0.4913,0.4355,0.0791,0.0049</t>
-  </si>
-  <si>
-    <t>0.6399,0.1365,0.1523,0.0400</t>
-  </si>
-  <si>
-    <t>0.4516,0.5501,0.0357,0.0041</t>
-  </si>
-  <si>
-    <t>0.6065,0.2271,0.1010,0.0400</t>
-  </si>
-  <si>
-    <t>0.9821,0.0314,0.0003,0.0003</t>
-  </si>
-  <si>
-    <t>0.9861,0.0241,0.0002,0.0002</t>
-  </si>
-  <si>
-    <t>0.8813,0.1985,0.0014,0.0004</t>
-  </si>
-  <si>
-    <t>0.9886,0.0197,0.0002,0.0002</t>
-  </si>
-  <si>
-    <t>0.9886,0.0188,0.0002,0.0002</t>
-  </si>
-  <si>
-    <t>0.9594,0.0745,0.0005,0.0003</t>
-  </si>
-  <si>
-    <t>0.9946,0.0098,0.0001,0.0001</t>
-  </si>
-  <si>
-    <t>0.9919,0.0135,0.0002,0.0002</t>
-  </si>
-  <si>
-    <t>0.0869,0.7510,0.2383,0.0015</t>
-  </si>
-  <si>
-    <t>0.0372,0.1197,0.8860,0.0005</t>
-  </si>
-  <si>
-    <t>0.0992,0.0842,0.8016,0.0007</t>
-  </si>
-  <si>
-    <t>0.0062,0.3608,0.9338,0.0004</t>
-  </si>
-  <si>
-    <t>0.2956,0.4685,0.2243,0.0035</t>
-  </si>
-  <si>
-    <t>0.0001,0.9994,0.0031,0.0000</t>
-  </si>
-  <si>
-    <t>0.0014,0.9956,0.0157,0.0000</t>
-  </si>
-  <si>
-    <t>0.0636,0.9093,0.0419,0.0004</t>
-  </si>
-  <si>
-    <t>0.0010,0.9968,0.0140,0.0000</t>
-  </si>
-  <si>
-    <t>0.0004,0.9986,0.0072,0.0000</t>
-  </si>
-  <si>
-    <t>0.1445,0.2741,0.5824,0.0025</t>
-  </si>
-  <si>
-    <t>0.0735,0.0575,0.8649,0.0006</t>
-  </si>
-  <si>
-    <t>0.0163,0.0037,0.9849,0.0002</t>
-  </si>
-  <si>
-    <t>0.0130,0.0911,0.9540,0.0002</t>
-  </si>
-  <si>
-    <t>0.0246,0.0298,0.9574,0.0002</t>
-  </si>
-  <si>
-    <t>0.0194,0.0218,0.9666,0.0001</t>
-  </si>
-  <si>
-    <t>0.0008,0.0104,0.9981,0.0000</t>
-  </si>
-  <si>
-    <t>0.0141,0.9743,0.0313,0.0001</t>
-  </si>
-  <si>
-    <t>0.3327,0.5887,0.1025,0.0031</t>
-  </si>
-  <si>
-    <t>0.0003,0.0340,0.9987,0.0000</t>
-  </si>
-  <si>
-    <t>0.0017,0.9622,0.4811,0.0000</t>
-  </si>
-  <si>
-    <t>0.2434,0.7380,0.0433,0.0015</t>
-  </si>
-  <si>
-    <t>0.0823,0.5230,0.5743,0.0022</t>
-  </si>
-  <si>
-    <t>0.2087,0.7716,0.0367,0.0007</t>
-  </si>
-  <si>
-    <t>0.0097,0.9598,0.1184,0.0001</t>
-  </si>
-  <si>
-    <t>0.0003,0.7948,0.9689,0.0000</t>
-  </si>
-  <si>
-    <t>0.0032,0.0187,0.9934,0.0001</t>
-  </si>
-  <si>
-    <t>0.0051,0.1060,0.9762,0.0001</t>
-  </si>
-  <si>
-    <t>0.0151,0.0297,0.9698,0.0002</t>
-  </si>
-  <si>
-    <t>0.0046,0.5069,0.9004,0.0001</t>
-  </si>
-  <si>
-    <t>0.0004,0.9713,0.6681,0.0000</t>
-  </si>
-  <si>
-    <t>0.0011,0.0499,0.9952,0.0000</t>
-  </si>
-  <si>
-    <t>0.4350,0.1830,0.3328,0.0277</t>
-  </si>
-  <si>
-    <t>0.0009,0.9951,0.0343,0.0000</t>
-  </si>
-  <si>
-    <t>0.0009,0.9829,0.3426,0.0000</t>
-  </si>
-  <si>
-    <t>0.0003,0.9958,0.1310,0.0000</t>
-  </si>
-  <si>
-    <t>0.0013,0.0321,0.9955,0.0000</t>
-  </si>
-  <si>
-    <t>0.0006,0.0914,0.9951,0.0000</t>
-  </si>
-  <si>
-    <t>0.0065,0.0151,0.9886,0.0001</t>
-  </si>
-  <si>
-    <t>0.0090,0.0103,0.9870,0.0001</t>
-  </si>
-  <si>
-    <t>0.0004,0.0289,0.9983,0.0000</t>
-  </si>
-  <si>
-    <t>0.0083,0.0156,0.9858,0.0002</t>
-  </si>
-  <si>
-    <t>0.6200,0.4752,0.0069,0.0006</t>
-  </si>
-  <si>
-    <t>0.9100,0.1428,0.0015,0.0006</t>
-  </si>
-  <si>
-    <t>0.9246,0.1219,0.0013,0.0007</t>
-  </si>
-  <si>
-    <t>0.0050,0.0992,0.9835,0.0004</t>
-  </si>
-  <si>
-    <t>0.9352,0.0997,0.0013,0.0007</t>
-  </si>
-  <si>
-    <t>0.9442,0.0978,0.0009,0.0004</t>
-  </si>
-  <si>
-    <t>0.6081,0.4939,0.0054,0.0007</t>
-  </si>
-  <si>
-    <t>0.0001,0.9758,0.8950,0.0000</t>
-  </si>
-  <si>
-    <t>0.0005,0.2426,0.9931,0.0000</t>
-  </si>
-  <si>
-    <t>0.0011,0.0447,0.9952,0.0000</t>
-  </si>
-  <si>
-    <t>0.0001,0.8122,0.9910,0.0000</t>
-  </si>
-  <si>
-    <t>0.0004,0.0155,0.9987,0.0000</t>
-  </si>
-  <si>
-    <t>0.0074,0.9628,0.1540,0.0001</t>
-  </si>
-  <si>
-    <t>0.0001,0.9997,0.0033,0.0000</t>
-  </si>
-  <si>
-    <t>0.2298,0.2219,0.5119,0.0016</t>
-  </si>
-  <si>
-    <t>0.1301,0.7591,0.1291,0.0012</t>
-  </si>
-  <si>
-    <t>0.0002,0.0894,0.9986,0.0000</t>
-  </si>
-  <si>
-    <t>0.0000,0.9513,0.9685,0.0000</t>
-  </si>
-  <si>
-    <t>0.0002,0.9197,0.9476,0.0000</t>
-  </si>
-  <si>
-    <t>0.0001,0.9711,0.8638,0.0000</t>
-  </si>
-  <si>
-    <t>0.0001,0.9537,0.9299,0.0000</t>
-  </si>
-  <si>
-    <t>0.5364,0.0658,0.0948,0.1960</t>
-  </si>
-  <si>
-    <t>0.0472,0.1186,0.0067,0.9464</t>
-  </si>
-  <si>
-    <t>0.0363,0.0193,0.0420,0.9513</t>
-  </si>
-  <si>
-    <t>0.5509,0.0372,0.0263,0.2825</t>
-  </si>
-  <si>
-    <t>0.6787,0.1251,0.0668,0.0582</t>
-  </si>
-  <si>
-    <t>0.0763,0.0386,0.0249,0.9189</t>
-  </si>
-  <si>
-    <t>0.0001,0.9644,0.9257,0.0000</t>
-  </si>
-  <si>
-    <t>0.0001,0.8296,0.9851,0.0000</t>
-  </si>
-  <si>
-    <t>0.0003,0.6718,0.9846,0.0000</t>
-  </si>
-  <si>
-    <t>0.0001,0.9253,0.9473,0.0000</t>
-  </si>
-  <si>
-    <t>0.0000,0.9617,0.9724,0.0000</t>
-  </si>
-  <si>
-    <t>0.0001,0.9061,0.9835,0.0000</t>
-  </si>
-  <si>
-    <t>0.9501,0.0923,0.0006,0.0002</t>
-  </si>
-  <si>
-    <t>0.9408,0.1010,0.0009,0.0004</t>
-  </si>
-  <si>
-    <t>0.7488,0.3716,0.0023,0.0003</t>
-  </si>
-  <si>
-    <t>0.9877,0.0204,0.0002,0.0003</t>
-  </si>
-  <si>
-    <t>0.8860,0.1698,0.0024,0.0008</t>
-  </si>
-  <si>
-    <t>0.9720,0.0546,0.0003,0.0002</t>
-  </si>
-  <si>
-    <t>0.9644,0.0597,0.0007,0.0004</t>
-  </si>
-  <si>
-    <t>0.8656,0.2129,0.0018,0.0004</t>
-  </si>
-  <si>
-    <t>0.9960,0.0068,0.0001,0.0001</t>
-  </si>
-  <si>
-    <t>0.9898,0.0179,0.0002,0.0002</t>
-  </si>
-  <si>
-    <t>0.9934,0.0115,0.0001,0.0001</t>
-  </si>
-  <si>
-    <t>0.9855,0.0257,0.0002,0.0002</t>
-  </si>
-  <si>
-    <t>0.9881,0.0224,0.0002,0.0001</t>
-  </si>
-  <si>
-    <t>0.9766,0.0423,0.0004,0.0002</t>
-  </si>
-  <si>
-    <t>0.9850,0.0256,0.0003,0.0002</t>
-  </si>
-  <si>
-    <t>0.9818,0.0309,0.0003,0.0003</t>
-  </si>
-  <si>
-    <t>0.0004,0.0038,0.9992,0.0000</t>
-  </si>
-  <si>
-    <t>0.0156,0.0239,0.9737,0.0003</t>
-  </si>
-  <si>
-    <t>0.5435,0.0990,0.3542,0.0066</t>
-  </si>
-  <si>
-    <t>0.0019,0.0478,0.9926,0.0000</t>
-  </si>
-  <si>
-    <t>0.0128,0.9770,0.0220,0.0001</t>
-  </si>
-  <si>
-    <t>0.0036,0.9920,0.0132,0.0000</t>
-  </si>
-  <si>
-    <t>0.0156,0.9789,0.0108,0.0001</t>
-  </si>
-  <si>
-    <t>0.0053,0.9905,0.0115,0.0000</t>
-  </si>
-  <si>
-    <t>0.0028,0.9929,0.0158,0.0000</t>
-  </si>
-  <si>
-    <t>0.0015,0.9962,0.0080,0.0000</t>
-  </si>
-  <si>
-    <t>0.0293,0.9598,0.0200,0.0001</t>
-  </si>
-  <si>
-    <t>0.0747,0.3443,0.6632,0.0011</t>
-  </si>
-  <si>
-    <t>0.2114,0.0458,0.7359,0.0022</t>
-  </si>
-  <si>
-    <t>0.1549,0.3531,0.5179,0.0030</t>
-  </si>
-  <si>
-    <t>0.1402,0.1240,0.7209,0.0017</t>
-  </si>
-  <si>
-    <t>0.1983,0.4013,0.4321,0.0082</t>
-  </si>
-  <si>
-    <t>0.0006,0.9974,0.0151,0.0000</t>
-  </si>
-  <si>
-    <t>0.0001,0.9989,0.0147,0.0000</t>
-  </si>
-  <si>
-    <t>0.0050,0.9856,0.0359,0.0001</t>
-  </si>
-  <si>
-    <t>0.0000,0.9904,0.9454,0.0000</t>
-  </si>
-  <si>
-    <t>0.0044,0.9879,0.0275,0.0000</t>
-  </si>
-  <si>
-    <t>0.1533,0.8210,0.0353,0.0005</t>
-  </si>
-  <si>
-    <t>0.2399,0.7562,0.0309,0.0007</t>
-  </si>
-  <si>
-    <t>0.6849,0.3900,0.0062,0.0005</t>
-  </si>
-  <si>
-    <t>0.9494,0.0821,0.0010,0.0005</t>
-  </si>
-  <si>
-    <t>0.9709,0.0502,0.0005,0.0003</t>
-  </si>
-  <si>
-    <t>0.9288,0.1074,0.0016,0.0008</t>
-  </si>
-  <si>
-    <t>0.9424,0.0981,0.0010,0.0004</t>
-  </si>
-  <si>
-    <t>0.3360,0.6741,0.0212,0.0007</t>
-  </si>
-  <si>
-    <t>0.7897,0.2964,0.0038,0.0009</t>
-  </si>
-  <si>
-    <t>0.8820,0.1721,0.0029,0.0007</t>
-  </si>
-  <si>
-    <t>0.0001,0.8021,0.9861,0.0000</t>
-  </si>
-  <si>
-    <t>0.0003,0.6304,0.9803,0.0000</t>
-  </si>
-  <si>
-    <t>0.0015,0.1156,0.9909,0.0000</t>
-  </si>
-  <si>
-    <t>0.0057,0.1024,0.9734,0.0001</t>
-  </si>
-  <si>
-    <t>0.4472,0.1993,0.3214,0.0076</t>
-  </si>
-  <si>
-    <t>0.2457,0.5920,0.1630,0.0024</t>
-  </si>
-  <si>
-    <t>0.0149,0.0613,0.9607,0.0002</t>
-  </si>
-  <si>
-    <t>0.2279,0.5957,0.2031,0.0042</t>
-  </si>
-  <si>
-    <t>0.7170,0.1005,0.1064,0.0360</t>
-  </si>
-  <si>
-    <t>0.0029,0.0181,0.0060,0.9964</t>
-  </si>
-  <si>
-    <t>0.0236,0.0808,0.0082,0.9780</t>
-  </si>
-  <si>
-    <t>0.3400,0.1569,0.0413,0.4579</t>
-  </si>
-  <si>
-    <t>0.0000,0.9881,0.9571,0.0000</t>
-  </si>
-  <si>
-    <t>0.8727,0.1808,0.0026,0.0008</t>
-  </si>
-  <si>
-    <t>0.1380,0.8389,0.0333,0.0007</t>
-  </si>
-  <si>
-    <t>0.7126,0.3273,0.0120,0.0016</t>
-  </si>
-  <si>
-    <t>0.1257,0.8521,0.0319,0.0006</t>
-  </si>
-  <si>
-    <t>0.8767,0.1644,0.0039,0.0012</t>
-  </si>
-  <si>
-    <t>0.6918,0.2058,0.0813,0.0104</t>
-  </si>
-  <si>
-    <t>0.6984,0.3283,0.0157,0.0020</t>
-  </si>
-  <si>
-    <t>0.1321,0.2024,0.7033,0.0074</t>
-  </si>
-  <si>
-    <t>0.7528,0.1313,0.0833,0.0057</t>
-  </si>
-  <si>
-    <t>0.7901,0.2039,0.0182,0.0035</t>
-  </si>
-  <si>
-    <t>0.0456,0.9282,0.0395,0.0003</t>
-  </si>
-  <si>
-    <t>0.5258,0.4419,0.0533,0.0040</t>
-  </si>
-  <si>
-    <t>0.1908,0.7651,0.0572,0.0010</t>
-  </si>
-  <si>
-    <t>0.0687,0.8414,0.1415,0.0010</t>
-  </si>
-  <si>
-    <t>0.0813,0.8310,0.1418,0.0009</t>
-  </si>
-  <si>
-    <t>0.1568,0.8109,0.0490,0.0013</t>
-  </si>
-  <si>
-    <t>0.9734,0.0417,0.0007,0.0005</t>
-  </si>
-  <si>
-    <t>0.9886,0.0174,0.0002,0.0003</t>
-  </si>
-  <si>
-    <t>0.9367,0.0967,0.0013,0.0007</t>
-  </si>
-  <si>
-    <t>0.9890,0.0159,0.0003,0.0003</t>
-  </si>
-  <si>
-    <t>0.9699,0.0460,0.0008,0.0005</t>
-  </si>
-  <si>
-    <t>0.9533,0.0739,0.0011,0.0006</t>
-  </si>
-  <si>
-    <t>0.9628,0.0593,0.0008,0.0006</t>
-  </si>
-  <si>
-    <t>0.9791,0.0318,0.0005,0.0004</t>
-  </si>
-  <si>
-    <t>0.0249,0.9646,0.0182,0.0002</t>
-  </si>
-  <si>
-    <t>0.2306,0.7698,0.0260,0.0008</t>
-  </si>
-  <si>
-    <t>0.1499,0.8198,0.0412,0.0006</t>
-  </si>
-  <si>
-    <t>0.4274,0.5344,0.0651,0.0025</t>
-  </si>
-  <si>
-    <t>0.2424,0.7916,0.0108,0.0004</t>
-  </si>
-  <si>
-    <t>0.5307,0.4740,0.0299,0.0027</t>
-  </si>
-  <si>
-    <t>0.4173,0.6536,0.0101,0.0006</t>
-  </si>
-  <si>
-    <t>0.4530,0.5832,0.0210,0.0013</t>
-  </si>
-  <si>
-    <t>0.0002,0.0320,0.9993,0.0000</t>
-  </si>
-  <si>
-    <t>0.5896,0.4863,0.0099,0.0013</t>
-  </si>
-  <si>
-    <t>0.0004,0.0036,0.9993,0.0000</t>
-  </si>
-  <si>
-    <t>0.0010,0.2239,0.9892,0.0001</t>
-  </si>
-  <si>
-    <t>0.0249,0.0273,0.9565,0.0002</t>
-  </si>
-  <si>
-    <t>0.0014,0.0594,0.9936,0.0000</t>
-  </si>
-  <si>
-    <t>0.0006,0.0152,0.9984,0.0000</t>
-  </si>
-  <si>
-    <t>0.0012,0.0145,0.9973,0.0000</t>
-  </si>
-  <si>
-    <t>0.0052,0.0262,0.9890,0.0001</t>
-  </si>
-  <si>
-    <t>0.1111,0.2503,0.6660,0.0019</t>
-  </si>
-  <si>
-    <t>0.0359,0.3845,0.7508,0.0006</t>
-  </si>
-  <si>
-    <t>0.0762,0.7499,0.2554,0.0011</t>
-  </si>
-  <si>
-    <t>0.0609,0.3952,0.6323,0.0010</t>
-  </si>
-  <si>
-    <t>0.0116,0.5937,0.8110,0.0003</t>
-  </si>
-  <si>
-    <t>0.0873,0.5193,0.5109,0.0023</t>
-  </si>
-  <si>
-    <t>0.1598,0.2448,0.5975,0.0022</t>
-  </si>
-  <si>
-    <t>0.0307,0.9132,0.1364,0.0006</t>
-  </si>
-  <si>
-    <t>0.0295,0.9672,0.0101,0.0001</t>
-  </si>
-  <si>
-    <t>0.0294,0.9653,0.0122,0.0001</t>
-  </si>
-  <si>
-    <t>0.1097,0.8877,0.0165,0.0002</t>
-  </si>
-  <si>
-    <t>0.5113,0.6047,0.0037,0.0003</t>
-  </si>
-  <si>
-    <t>0.2073,0.8267,0.0095,0.0004</t>
-  </si>
-  <si>
-    <t>0.0226,0.9306,0.1195,0.0004</t>
-  </si>
-  <si>
-    <t>0.3754,0.1139,0.4905,0.0037</t>
-  </si>
-  <si>
-    <t>0.3291,0.2406,0.4077,0.0065</t>
-  </si>
-  <si>
-    <t>0.1252,0.3263,0.5900,0.0030</t>
-  </si>
-  <si>
-    <t>0.3326,0.1166,0.5366,0.0036</t>
-  </si>
-  <si>
-    <t>0.0043,0.0486,0.9875,0.0001</t>
-  </si>
-  <si>
-    <t>0.0005,0.1355,0.9955,0.0000</t>
-  </si>
-  <si>
-    <t>0.0007,0.1767,0.9934,0.0000</t>
-  </si>
-  <si>
-    <t>0.0012,0.0396,0.9953,0.0000</t>
-  </si>
-  <si>
-    <t>0.0018,0.5429,0.9519,0.0002</t>
-  </si>
-  <si>
-    <t>0.9639,0.0608,0.0006,0.0004</t>
-  </si>
-  <si>
-    <t>0.6640,0.4552,0.0034,0.0005</t>
-  </si>
-  <si>
-    <t>0.8562,0.2228,0.0021,0.0005</t>
-  </si>
-  <si>
-    <t>0.8505,0.2415,0.0017,0.0004</t>
-  </si>
-  <si>
-    <t>0.9290,0.1227,0.0010,0.0004</t>
-  </si>
-  <si>
-    <t>0.9031,0.1529,0.0017,0.0005</t>
-  </si>
-  <si>
-    <t>0.9511,0.0823,0.0009,0.0004</t>
-  </si>
-  <si>
-    <t>0.9726,0.0445,0.0006,0.0004</t>
-  </si>
-  <si>
-    <t>0.0470,0.0706,0.8996,0.0005</t>
-  </si>
-  <si>
-    <t>0.0712,0.8436,0.1356,0.0010</t>
-  </si>
-  <si>
-    <t>0.5060,0.4483,0.0620,0.0031</t>
-  </si>
-  <si>
-    <t>0.0003,0.0081,0.9992,0.0000</t>
-  </si>
-  <si>
-    <t>0.0004,0.0082,0.9989,0.0000</t>
-  </si>
-  <si>
-    <t>0.0023,0.2049,0.9767,0.0001</t>
-  </si>
-  <si>
-    <t>0.0000,0.0029,0.9999,0.0000</t>
-  </si>
-  <si>
-    <t>0.0069,0.0982,0.9694,0.0001</t>
-  </si>
-  <si>
-    <t>0.0004,0.0047,0.9992,0.0000</t>
-  </si>
-  <si>
-    <t>0.0050,0.0067,0.9934,0.0000</t>
-  </si>
-  <si>
-    <t>0.0021,0.3799,0.9662,0.0001</t>
-  </si>
-  <si>
-    <t>0.0976,0.5094,0.4466,0.0022</t>
-  </si>
-  <si>
-    <t>0.4142,0.0485,0.5567,0.0025</t>
-  </si>
-  <si>
-    <t>0.1718,0.1317,0.7001,0.0031</t>
-  </si>
-  <si>
-    <t>0.9750,0.0448,0.0004,0.0003</t>
-  </si>
-  <si>
-    <t>0.9604,0.0706,0.0006,0.0003</t>
-  </si>
-  <si>
-    <t>0.9753,0.0463,0.0004,0.0002</t>
-  </si>
-  <si>
-    <t>0.9629,0.0653,0.0007,0.0003</t>
-  </si>
-  <si>
-    <t>0.9688,0.0499,0.0006,0.0005</t>
-  </si>
-  <si>
-    <t>0.8469,0.2272,0.0029,0.0006</t>
-  </si>
-  <si>
-    <t>0.9673,0.0581,0.0006,0.0003</t>
-  </si>
-  <si>
-    <t>0.9625,0.0587,0.0009,0.0006</t>
-  </si>
-  <si>
-    <t>0.0044,0.0564,0.9834,0.0001</t>
-  </si>
-  <si>
-    <t>0.0001,0.0263,0.9994,0.0000</t>
-  </si>
-  <si>
-    <t>0.0006,0.1434,0.9938,0.0000</t>
-  </si>
-  <si>
-    <t>0.0055,0.5870,0.8713,0.0002</t>
-  </si>
-  <si>
-    <t>0.0009,0.0062,0.9982,0.0000</t>
-  </si>
-  <si>
-    <t>0.0541,0.0682,0.8895,0.0005</t>
-  </si>
-  <si>
-    <t>0.0523,0.0854,0.8707,0.0004</t>
-  </si>
-  <si>
-    <t>0.0044,0.0149,0.9916,0.0001</t>
-  </si>
-  <si>
-    <t>0.7226,0.1901,0.0677,0.0065</t>
-  </si>
-  <si>
-    <t>0.5105,0.1839,0.1751,0.0873</t>
-  </si>
-  <si>
-    <t>0.5644,0.0420,0.0229,0.2789</t>
-  </si>
-  <si>
-    <t>0.0823,0.0488,0.0053,0.9172</t>
-  </si>
-  <si>
-    <t>0.0438,0.0922,0.0043,0.9556</t>
-  </si>
-  <si>
-    <t>0.3764,0.5036,0.1109,0.0064</t>
+    <t>0,0,0,0</t>
+  </si>
+  <si>
+    <t>1,1,0,0</t>
+  </si>
+  <si>
+    <t>0.3677,0.6082,0.0474,0.0047</t>
+  </si>
+  <si>
+    <t>0.7181,0.1132,0.1189,0.0228</t>
+  </si>
+  <si>
+    <t>0.5719,0.4486,0.0186,0.0059</t>
+  </si>
+  <si>
+    <t>0.5273,0.3570,0.0730,0.0353</t>
+  </si>
+  <si>
+    <t>0.9832,0.0318,0.0002,0.0002</t>
+  </si>
+  <si>
+    <t>0.9835,0.0307,0.0003,0.0002</t>
+  </si>
+  <si>
+    <t>0.9299,0.1224,0.0010,0.0003</t>
+  </si>
+  <si>
+    <t>0.9759,0.0409,0.0005,0.0003</t>
+  </si>
+  <si>
+    <t>0.9900,0.0169,0.0002,0.0002</t>
+  </si>
+  <si>
+    <t>0.9618,0.0682,0.0005,0.0003</t>
+  </si>
+  <si>
+    <t>0.9946,0.0097,0.0001,0.0001</t>
+  </si>
+  <si>
+    <t>0.9805,0.0348,0.0003,0.0002</t>
+  </si>
+  <si>
+    <t>0.1136,0.7965,0.1159,0.0022</t>
+  </si>
+  <si>
+    <t>0.0166,0.0577,0.9597,0.0002</t>
+  </si>
+  <si>
+    <t>0.0630,0.1354,0.8244,0.0005</t>
+  </si>
+  <si>
+    <t>0.0079,0.3021,0.9265,0.0002</t>
+  </si>
+  <si>
+    <t>0.1817,0.6152,0.2288,0.0025</t>
+  </si>
+  <si>
+    <t>0.0002,0.9991,0.0048,0.0000</t>
+  </si>
+  <si>
+    <t>0.0011,0.9957,0.0230,0.0000</t>
+  </si>
+  <si>
+    <t>0.0674,0.9117,0.0336,0.0004</t>
+  </si>
+  <si>
+    <t>0.0014,0.9961,0.0109,0.0000</t>
+  </si>
+  <si>
+    <t>0.0003,0.9985,0.0101,0.0000</t>
+  </si>
+  <si>
+    <t>0.2345,0.0836,0.6734,0.0019</t>
+  </si>
+  <si>
+    <t>0.0841,0.0276,0.8859,0.0006</t>
+  </si>
+  <si>
+    <t>0.0033,0.0061,0.9953,0.0000</t>
+  </si>
+  <si>
+    <t>0.0492,0.0263,0.9250,0.0002</t>
+  </si>
+  <si>
+    <t>0.0279,0.0104,0.9686,0.0001</t>
+  </si>
+  <si>
+    <t>0.0504,0.0296,0.9232,0.0003</t>
+  </si>
+  <si>
+    <t>0.0022,0.0020,0.9973,0.0001</t>
+  </si>
+  <si>
+    <t>0.0180,0.9726,0.0218,0.0002</t>
+  </si>
+  <si>
+    <t>0.1713,0.7381,0.1022,0.0014</t>
+  </si>
+  <si>
+    <t>0.0003,0.0614,0.9980,0.0001</t>
+  </si>
+  <si>
+    <t>0.0007,0.9359,0.7711,0.0000</t>
+  </si>
+  <si>
+    <t>0.3505,0.5854,0.0897,0.0034</t>
+  </si>
+  <si>
+    <t>0.0772,0.4160,0.6573,0.0020</t>
+  </si>
+  <si>
+    <t>0.1975,0.7847,0.0386,0.0008</t>
+  </si>
+  <si>
+    <t>0.0058,0.9840,0.0353,0.0000</t>
+  </si>
+  <si>
+    <t>0.0009,0.6963,0.9527,0.0001</t>
+  </si>
+  <si>
+    <t>0.0023,0.0105,0.9954,0.0002</t>
+  </si>
+  <si>
+    <t>0.0015,0.1309,0.9900,0.0000</t>
+  </si>
+  <si>
+    <t>0.0125,0.0053,0.9864,0.0002</t>
+  </si>
+  <si>
+    <t>0.0031,0.0491,0.9892,0.0000</t>
+  </si>
+  <si>
+    <t>0.0001,0.9825,0.7719,0.0000</t>
+  </si>
+  <si>
+    <t>0.0012,0.0367,0.9956,0.0000</t>
+  </si>
+  <si>
+    <t>0.4743,0.2774,0.2110,0.0239</t>
+  </si>
+  <si>
+    <t>0.0017,0.9929,0.0283,0.0001</t>
+  </si>
+  <si>
+    <t>0.0005,0.9956,0.0855,0.0000</t>
+  </si>
+  <si>
+    <t>0.0002,0.9969,0.1318,0.0000</t>
+  </si>
+  <si>
+    <t>0.0014,0.0267,0.9956,0.0000</t>
+  </si>
+  <si>
+    <t>0.0004,0.0480,0.9976,0.0000</t>
+  </si>
+  <si>
+    <t>0.0312,0.0565,0.9271,0.0003</t>
+  </si>
+  <si>
+    <t>0.0069,0.0059,0.9915,0.0001</t>
+  </si>
+  <si>
+    <t>0.0014,0.0108,0.9971,0.0000</t>
+  </si>
+  <si>
+    <t>0.0038,0.0138,0.9927,0.0001</t>
+  </si>
+  <si>
+    <t>0.5107,0.5739,0.0089,0.0008</t>
+  </si>
+  <si>
+    <t>0.7995,0.2784,0.0046,0.0009</t>
+  </si>
+  <si>
+    <t>0.9128,0.1288,0.0025,0.0008</t>
+  </si>
+  <si>
+    <t>0.0040,0.1304,0.9832,0.0002</t>
+  </si>
+  <si>
+    <t>0.9387,0.0944,0.0013,0.0007</t>
+  </si>
+  <si>
+    <t>0.9291,0.1255,0.0009,0.0004</t>
+  </si>
+  <si>
+    <t>0.3991,0.6857,0.0068,0.0005</t>
+  </si>
+  <si>
+    <t>0.0001,0.9487,0.9571,0.0000</t>
+  </si>
+  <si>
+    <t>0.0008,0.0869,0.9952,0.0000</t>
+  </si>
+  <si>
+    <t>0.0005,0.3743,0.9875,0.0000</t>
+  </si>
+  <si>
+    <t>0.0000,0.9501,0.9838,0.0000</t>
+  </si>
+  <si>
+    <t>0.0006,0.0095,0.9988,0.0000</t>
+  </si>
+  <si>
+    <t>0.0048,0.9749,0.1280,0.0001</t>
+  </si>
+  <si>
+    <t>0.0000,0.9998,0.0038,0.0000</t>
+  </si>
+  <si>
+    <t>0.1637,0.1285,0.7042,0.0014</t>
+  </si>
+  <si>
+    <t>0.0769,0.8748,0.0689,0.0010</t>
+  </si>
+  <si>
+    <t>0.0002,0.0643,0.9987,0.0000</t>
+  </si>
+  <si>
+    <t>0.0001,0.9220,0.9664,0.0000</t>
+  </si>
+  <si>
+    <t>0.0004,0.9177,0.8606,0.0000</t>
+  </si>
+  <si>
+    <t>0.0001,0.9851,0.7390,0.0000</t>
+  </si>
+  <si>
+    <t>0.0000,0.9880,0.9499,0.0000</t>
+  </si>
+  <si>
+    <t>0.6236,0.0504,0.2824,0.0469</t>
+  </si>
+  <si>
+    <t>0.0153,0.1407,0.0038,0.9810</t>
+  </si>
+  <si>
+    <t>0.0904,0.0896,0.0212,0.8980</t>
+  </si>
+  <si>
+    <t>0.3801,0.0592,0.0146,0.5303</t>
+  </si>
+  <si>
+    <t>0.4768,0.0633,0.0234,0.3571</t>
+  </si>
+  <si>
+    <t>0.0280,0.0149,0.0744,0.9534</t>
+  </si>
+  <si>
+    <t>0.0001,0.9186,0.9692,0.0000</t>
+  </si>
+  <si>
+    <t>0.0002,0.7504,0.9836,0.0000</t>
+  </si>
+  <si>
+    <t>0.0001,0.8195,0.9826,0.0000</t>
+  </si>
+  <si>
+    <t>0.0002,0.8427,0.9633,0.0000</t>
+  </si>
+  <si>
+    <t>0.0001,0.8554,0.9892,0.0000</t>
+  </si>
+  <si>
+    <t>0.0002,0.8006,0.9794,0.0000</t>
+  </si>
+  <si>
+    <t>0.9649,0.0678,0.0004,0.0002</t>
+  </si>
+  <si>
+    <t>0.8993,0.1678,0.0014,0.0004</t>
+  </si>
+  <si>
+    <t>0.8308,0.2672,0.0020,0.0003</t>
+  </si>
+  <si>
+    <t>0.9823,0.0302,0.0003,0.0003</t>
+  </si>
+  <si>
+    <t>0.9099,0.1354,0.0020,0.0007</t>
+  </si>
+  <si>
+    <t>0.9771,0.0436,0.0003,0.0002</t>
+  </si>
+  <si>
+    <t>0.9617,0.0592,0.0009,0.0006</t>
+  </si>
+  <si>
+    <t>0.9184,0.1410,0.0010,0.0003</t>
+  </si>
+  <si>
+    <t>0.9955,0.0074,0.0001,0.0001</t>
+  </si>
+  <si>
+    <t>0.9915,0.0155,0.0001,0.0001</t>
+  </si>
+  <si>
+    <t>0.9954,0.0077,0.0001,0.0001</t>
+  </si>
+  <si>
+    <t>0.9782,0.0424,0.0003,0.0002</t>
+  </si>
+  <si>
+    <t>0.9911,0.0153,0.0001,0.0002</t>
+  </si>
+  <si>
+    <t>0.9867,0.0250,0.0002,0.0002</t>
+  </si>
+  <si>
+    <t>0.9888,0.0194,0.0002,0.0002</t>
+  </si>
+  <si>
+    <t>0.9923,0.0128,0.0002,0.0002</t>
+  </si>
+  <si>
+    <t>0.0006,0.0012,0.9993,0.0000</t>
+  </si>
+  <si>
+    <t>0.0092,0.0468,0.9766,0.0001</t>
+  </si>
+  <si>
+    <t>0.4860,0.0694,0.4510,0.0036</t>
+  </si>
+  <si>
+    <t>0.0105,0.0253,0.9798,0.0001</t>
+  </si>
+  <si>
+    <t>0.0125,0.9780,0.0197,0.0001</t>
+  </si>
+  <si>
+    <t>0.0057,0.9879,0.0170,0.0000</t>
+  </si>
+  <si>
+    <t>0.0417,0.9517,0.0163,0.0002</t>
+  </si>
+  <si>
+    <t>0.0111,0.9829,0.0139,0.0001</t>
+  </si>
+  <si>
+    <t>0.0054,0.9877,0.0201,0.0000</t>
+  </si>
+  <si>
+    <t>0.0021,0.9950,0.0101,0.0000</t>
+  </si>
+  <si>
+    <t>0.0621,0.9239,0.0235,0.0003</t>
+  </si>
+  <si>
+    <t>0.0944,0.2949,0.6714,0.0014</t>
+  </si>
+  <si>
+    <t>0.2379,0.0216,0.7617,0.0008</t>
+  </si>
+  <si>
+    <t>0.0501,0.8083,0.2478,0.0010</t>
+  </si>
+  <si>
+    <t>0.2388,0.1365,0.5974,0.0031</t>
+  </si>
+  <si>
+    <t>0.3778,0.2784,0.3232,0.0118</t>
+  </si>
+  <si>
+    <t>0.0005,0.9967,0.0317,0.0000</t>
+  </si>
+  <si>
+    <t>0.0002,0.9971,0.0958,0.0000</t>
+  </si>
+  <si>
+    <t>0.0017,0.9945,0.0161,0.0001</t>
+  </si>
+  <si>
+    <t>0.0000,0.9906,0.9441,0.0000</t>
+  </si>
+  <si>
+    <t>0.0055,0.9870,0.0237,0.0000</t>
+  </si>
+  <si>
+    <t>0.1545,0.8275,0.0300,0.0004</t>
+  </si>
+  <si>
+    <t>0.1878,0.8057,0.0289,0.0006</t>
+  </si>
+  <si>
+    <t>0.3529,0.6939,0.0072,0.0003</t>
+  </si>
+  <si>
+    <t>0.8546,0.2248,0.0020,0.0006</t>
+  </si>
+  <si>
+    <t>0.9817,0.0305,0.0003,0.0003</t>
+  </si>
+  <si>
+    <t>0.8780,0.1761,0.0024,0.0009</t>
+  </si>
+  <si>
+    <t>0.8785,0.1878,0.0020,0.0006</t>
+  </si>
+  <si>
+    <t>0.4287,0.6064,0.0153,0.0010</t>
+  </si>
+  <si>
+    <t>0.9813,0.0324,0.0003,0.0003</t>
+  </si>
+  <si>
+    <t>0.8515,0.2184,0.0033,0.0007</t>
+  </si>
+  <si>
+    <t>0.0001,0.7842,0.9878,0.0000</t>
+  </si>
+  <si>
+    <t>0.0001,0.8394,0.9881,0.0000</t>
+  </si>
+  <si>
+    <t>0.0009,0.2802,0.9880,0.0000</t>
+  </si>
+  <si>
+    <t>0.0013,0.1932,0.9859,0.0000</t>
+  </si>
+  <si>
+    <t>0.5933,0.1406,0.2297,0.0053</t>
+  </si>
+  <si>
+    <t>0.3400,0.3202,0.3002,0.0034</t>
+  </si>
+  <si>
+    <t>0.2114,0.0214,0.7856,0.0019</t>
+  </si>
+  <si>
+    <t>0.0653,0.7967,0.2389,0.0011</t>
+  </si>
+  <si>
+    <t>0.7861,0.0921,0.0535,0.0286</t>
+  </si>
+  <si>
+    <t>0.0033,0.0073,0.0118,0.9956</t>
+  </si>
+  <si>
+    <t>0.0883,0.1290,0.0263,0.8906</t>
+  </si>
+  <si>
+    <t>0.5842,0.0566,0.1018,0.1428</t>
+  </si>
+  <si>
+    <t>0.0000,0.9808,0.9807,0.0000</t>
+  </si>
+  <si>
+    <t>0.9023,0.1380,0.0023,0.0009</t>
+  </si>
+  <si>
+    <t>0.1443,0.8452,0.0258,0.0011</t>
+  </si>
+  <si>
+    <t>0.8252,0.2246,0.0057,0.0014</t>
+  </si>
+  <si>
+    <t>0.1679,0.8139,0.0282,0.0005</t>
+  </si>
+  <si>
+    <t>0.5359,0.5344,0.0111,0.0011</t>
+  </si>
+  <si>
+    <t>0.6038,0.2804,0.1077,0.0080</t>
+  </si>
+  <si>
+    <t>0.8767,0.1513,0.0065,0.0015</t>
+  </si>
+  <si>
+    <t>0.0874,0.1160,0.8233,0.0043</t>
+  </si>
+  <si>
+    <t>0.8190,0.0894,0.0592,0.0057</t>
+  </si>
+  <si>
+    <t>0.6763,0.3007,0.0318,0.0055</t>
+  </si>
+  <si>
+    <t>0.0549,0.8700,0.1330,0.0005</t>
+  </si>
+  <si>
+    <t>0.4594,0.5029,0.0561,0.0027</t>
+  </si>
+  <si>
+    <t>0.1145,0.8590,0.0390,0.0006</t>
+  </si>
+  <si>
+    <t>0.0509,0.8278,0.2303,0.0007</t>
+  </si>
+  <si>
+    <t>0.1814,0.6648,0.1588,0.0014</t>
+  </si>
+  <si>
+    <t>0.2561,0.6874,0.0748,0.0018</t>
+  </si>
+  <si>
+    <t>0.9911,0.0148,0.0002,0.0002</t>
+  </si>
+  <si>
+    <t>0.9893,0.0166,0.0002,0.0003</t>
+  </si>
+  <si>
+    <t>0.9666,0.0539,0.0007,0.0004</t>
+  </si>
+  <si>
+    <t>0.9830,0.0262,0.0005,0.0003</t>
+  </si>
+  <si>
+    <t>0.9546,0.0761,0.0010,0.0004</t>
+  </si>
+  <si>
+    <t>0.8459,0.2236,0.0029,0.0008</t>
+  </si>
+  <si>
+    <t>0.8557,0.2158,0.0025,0.0008</t>
+  </si>
+  <si>
+    <t>0.9442,0.0835,0.0017,0.0007</t>
+  </si>
+  <si>
+    <t>0.0161,0.9734,0.0209,0.0001</t>
+  </si>
+  <si>
+    <t>0.1643,0.8346,0.0216,0.0006</t>
+  </si>
+  <si>
+    <t>0.1520,0.8233,0.0337,0.0005</t>
+  </si>
+  <si>
+    <t>0.0936,0.2524,0.7341,0.0015</t>
+  </si>
+  <si>
+    <t>0.1946,0.8338,0.0110,0.0003</t>
+  </si>
+  <si>
+    <t>0.4298,0.6005,0.0186,0.0017</t>
+  </si>
+  <si>
+    <t>0.4769,0.6006,0.0095,0.0006</t>
+  </si>
+  <si>
+    <t>0.4883,0.5830,0.0110,0.0011</t>
+  </si>
+  <si>
+    <t>0.0005,0.0273,0.9984,0.0000</t>
+  </si>
+  <si>
+    <t>0.5603,0.5297,0.0082,0.0009</t>
+  </si>
+  <si>
+    <t>0.0005,0.0209,0.9985,0.0000</t>
+  </si>
+  <si>
+    <t>0.0017,0.0497,0.9936,0.0001</t>
+  </si>
+  <si>
+    <t>0.0265,0.0312,0.9523,0.0001</t>
+  </si>
+  <si>
+    <t>0.0005,0.0868,0.9965,0.0000</t>
+  </si>
+  <si>
+    <t>0.0007,0.0175,0.9979,0.0000</t>
+  </si>
+  <si>
+    <t>0.0011,0.0082,0.9979,0.0000</t>
+  </si>
+  <si>
+    <t>0.0022,0.0269,0.9943,0.0000</t>
+  </si>
+  <si>
+    <t>0.0501,0.3031,0.7717,0.0010</t>
+  </si>
+  <si>
+    <t>0.2347,0.4169,0.3279,0.0028</t>
+  </si>
+  <si>
+    <t>0.0384,0.2896,0.8069,0.0005</t>
+  </si>
+  <si>
+    <t>0.0705,0.2544,0.7303,0.0008</t>
+  </si>
+  <si>
+    <t>0.0122,0.2650,0.9106,0.0003</t>
+  </si>
+  <si>
+    <t>0.0906,0.5411,0.4893,0.0021</t>
+  </si>
+  <si>
+    <t>0.2259,0.6241,0.1648,0.0029</t>
+  </si>
+  <si>
+    <t>0.0820,0.5551,0.4803,0.0014</t>
+  </si>
+  <si>
+    <t>0.0491,0.9471,0.0118,0.0001</t>
+  </si>
+  <si>
+    <t>0.0201,0.9750,0.0098,0.0001</t>
+  </si>
+  <si>
+    <t>0.1453,0.8676,0.0112,0.0002</t>
+  </si>
+  <si>
+    <t>0.3586,0.7091,0.0088,0.0005</t>
+  </si>
+  <si>
+    <t>0.1542,0.8663,0.0106,0.0003</t>
+  </si>
+  <si>
+    <t>0.0495,0.7789,0.3124,0.0009</t>
+  </si>
+  <si>
+    <t>0.3124,0.1957,0.4487,0.0029</t>
+  </si>
+  <si>
+    <t>0.5040,0.1605,0.3165,0.0099</t>
+  </si>
+  <si>
+    <t>0.0628,0.3578,0.6770,0.0010</t>
+  </si>
+  <si>
+    <t>0.1834,0.1418,0.6784,0.0032</t>
+  </si>
+  <si>
+    <t>0.0015,0.1680,0.9880,0.0001</t>
+  </si>
+  <si>
+    <t>0.0014,0.0375,0.9955,0.0000</t>
+  </si>
+  <si>
+    <t>0.0017,0.2976,0.9788,0.0001</t>
+  </si>
+  <si>
+    <t>0.0101,0.0298,0.9771,0.0001</t>
+  </si>
+  <si>
+    <t>0.0007,0.1909,0.9917,0.0001</t>
+  </si>
+  <si>
+    <t>0.9668,0.0546,0.0006,0.0005</t>
+  </si>
+  <si>
+    <t>0.7464,0.3738,0.0023,0.0004</t>
+  </si>
+  <si>
+    <t>0.9435,0.0930,0.0011,0.0005</t>
+  </si>
+  <si>
+    <t>0.8704,0.2251,0.0011,0.0003</t>
+  </si>
+  <si>
+    <t>0.9032,0.1581,0.0014,0.0005</t>
+  </si>
+  <si>
+    <t>0.9507,0.0810,0.0010,0.0004</t>
+  </si>
+  <si>
+    <t>0.9354,0.1024,0.0014,0.0006</t>
+  </si>
+  <si>
+    <t>0.9765,0.0388,0.0005,0.0004</t>
+  </si>
+  <si>
+    <t>0.0208,0.0971,0.9365,0.0003</t>
+  </si>
+  <si>
+    <t>0.0232,0.9589,0.0390,0.0002</t>
+  </si>
+  <si>
+    <t>0.6413,0.2812,0.0703,0.0046</t>
+  </si>
+  <si>
+    <t>0.0013,0.0043,0.9981,0.0000</t>
+  </si>
+  <si>
+    <t>0.0001,0.0093,0.9997,0.0000</t>
+  </si>
+  <si>
+    <t>0.0016,0.1337,0.9877,0.0000</t>
+  </si>
+  <si>
+    <t>0.0000,0.0053,0.9998,0.0000</t>
+  </si>
+  <si>
+    <t>0.0064,0.0304,0.9846,0.0001</t>
+  </si>
+  <si>
+    <t>0.0003,0.0037,0.9994,0.0000</t>
+  </si>
+  <si>
+    <t>0.0025,0.0288,0.9931,0.0000</t>
+  </si>
+  <si>
+    <t>0.0105,0.2984,0.9125,0.0003</t>
+  </si>
+  <si>
+    <t>0.0957,0.3941,0.5698,0.0023</t>
+  </si>
+  <si>
+    <t>0.3150,0.1536,0.4927,0.0033</t>
+  </si>
+  <si>
+    <t>0.2707,0.4019,0.3111,0.0049</t>
+  </si>
+  <si>
+    <t>0.9772,0.0397,0.0004,0.0003</t>
+  </si>
+  <si>
+    <t>0.9668,0.0623,0.0005,0.0002</t>
+  </si>
+  <si>
+    <t>0.9766,0.0437,0.0004,0.0002</t>
+  </si>
+  <si>
+    <t>0.8398,0.2561,0.0018,0.0003</t>
+  </si>
+  <si>
+    <t>0.9481,0.0942,0.0007,0.0003</t>
+  </si>
+  <si>
+    <t>0.8847,0.1875,0.0017,0.0004</t>
+  </si>
+  <si>
+    <t>0.9598,0.0747,0.0005,0.0003</t>
+  </si>
+  <si>
+    <t>0.9850,0.0244,0.0003,0.0003</t>
+  </si>
+  <si>
+    <t>0.0034,0.1558,0.9747,0.0001</t>
+  </si>
+  <si>
+    <t>0.0005,0.0197,0.9984,0.0000</t>
+  </si>
+  <si>
+    <t>0.0007,0.0923,0.9952,0.0000</t>
+  </si>
+  <si>
+    <t>0.0153,0.4783,0.8048,0.0003</t>
+  </si>
+  <si>
+    <t>0.0028,0.0093,0.9953,0.0001</t>
+  </si>
+  <si>
+    <t>0.0530,0.1156,0.8685,0.0009</t>
+  </si>
+  <si>
+    <t>0.0414,0.1970,0.8218,0.0005</t>
+  </si>
+  <si>
+    <t>0.0089,0.0116,0.9865,0.0001</t>
+  </si>
+  <si>
+    <t>0.5793,0.3368,0.0848,0.0052</t>
+  </si>
+  <si>
+    <t>0.5260,0.1509,0.2016,0.0981</t>
+  </si>
+  <si>
+    <t>0.6897,0.0555,0.0213,0.1463</t>
+  </si>
+  <si>
+    <t>0.0244,0.0295,0.0062,0.9792</t>
+  </si>
+  <si>
+    <t>0.0261,0.0599,0.0055,0.9772</t>
+  </si>
+  <si>
+    <t>0.2573,0.6368,0.1092,0.0058</t>
   </si>
 </sst>
 </file>
@@ -1953,10 +1959,10 @@
         <v>259</v>
       </c>
       <c r="C2" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1970,7 +1976,7 @@
         <v>259</v>
       </c>
       <c r="D3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1981,10 +1987,10 @@
         <v>259</v>
       </c>
       <c r="C4" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D4" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1998,7 +2004,7 @@
         <v>259</v>
       </c>
       <c r="D5" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2012,7 +2018,7 @@
         <v>259</v>
       </c>
       <c r="D6" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2026,7 +2032,7 @@
         <v>259</v>
       </c>
       <c r="D7" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2040,7 +2046,7 @@
         <v>259</v>
       </c>
       <c r="D8" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2054,7 +2060,7 @@
         <v>259</v>
       </c>
       <c r="D9" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2068,7 +2074,7 @@
         <v>259</v>
       </c>
       <c r="D10" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2082,7 +2088,7 @@
         <v>259</v>
       </c>
       <c r="D11" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2096,7 +2102,7 @@
         <v>259</v>
       </c>
       <c r="D12" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2110,7 +2116,7 @@
         <v>259</v>
       </c>
       <c r="D13" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -2124,7 +2130,7 @@
         <v>262</v>
       </c>
       <c r="D14" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2138,7 +2144,7 @@
         <v>261</v>
       </c>
       <c r="D15" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2152,7 +2158,7 @@
         <v>261</v>
       </c>
       <c r="D16" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2166,7 +2172,7 @@
         <v>261</v>
       </c>
       <c r="D17" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2177,10 +2183,10 @@
         <v>259</v>
       </c>
       <c r="C18" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -2194,7 +2200,7 @@
         <v>262</v>
       </c>
       <c r="D19" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2208,7 +2214,7 @@
         <v>262</v>
       </c>
       <c r="D20" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2222,7 +2228,7 @@
         <v>262</v>
       </c>
       <c r="D21" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -2236,7 +2242,7 @@
         <v>262</v>
       </c>
       <c r="D22" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -2250,7 +2256,7 @@
         <v>262</v>
       </c>
       <c r="D23" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -2264,7 +2270,7 @@
         <v>261</v>
       </c>
       <c r="D24" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -2278,7 +2284,7 @@
         <v>261</v>
       </c>
       <c r="D25" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2292,7 +2298,7 @@
         <v>261</v>
       </c>
       <c r="D26" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2306,7 +2312,7 @@
         <v>261</v>
       </c>
       <c r="D27" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2320,7 +2326,7 @@
         <v>261</v>
       </c>
       <c r="D28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2334,7 +2340,7 @@
         <v>261</v>
       </c>
       <c r="D29" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2348,7 +2354,7 @@
         <v>261</v>
       </c>
       <c r="D30" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -2362,7 +2368,7 @@
         <v>262</v>
       </c>
       <c r="D31" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -2376,7 +2382,7 @@
         <v>262</v>
       </c>
       <c r="D32" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -2390,7 +2396,7 @@
         <v>261</v>
       </c>
       <c r="D33" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -2401,10 +2407,10 @@
         <v>263</v>
       </c>
       <c r="C34" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D34" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -2418,7 +2424,7 @@
         <v>262</v>
       </c>
       <c r="D35" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -2429,10 +2435,10 @@
         <v>259</v>
       </c>
       <c r="C36" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D36" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -2446,7 +2452,7 @@
         <v>262</v>
       </c>
       <c r="D37" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -2460,7 +2466,7 @@
         <v>262</v>
       </c>
       <c r="D38" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -2474,7 +2480,7 @@
         <v>263</v>
       </c>
       <c r="D39" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -2488,7 +2494,7 @@
         <v>261</v>
       </c>
       <c r="D40" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -2502,7 +2508,7 @@
         <v>261</v>
       </c>
       <c r="D41" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -2516,7 +2522,7 @@
         <v>261</v>
       </c>
       <c r="D42" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -2527,10 +2533,10 @@
         <v>263</v>
       </c>
       <c r="C43" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D43" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -2544,7 +2550,7 @@
         <v>263</v>
       </c>
       <c r="D44" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -2558,7 +2564,7 @@
         <v>261</v>
       </c>
       <c r="D45" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -2569,10 +2575,10 @@
         <v>259</v>
       </c>
       <c r="C46" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D46" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -2586,7 +2592,7 @@
         <v>262</v>
       </c>
       <c r="D47" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -2600,7 +2606,7 @@
         <v>262</v>
       </c>
       <c r="D48" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -2614,7 +2620,7 @@
         <v>262</v>
       </c>
       <c r="D49" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -2628,7 +2634,7 @@
         <v>261</v>
       </c>
       <c r="D50" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -2642,7 +2648,7 @@
         <v>261</v>
       </c>
       <c r="D51" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -2656,7 +2662,7 @@
         <v>261</v>
       </c>
       <c r="D52" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -2670,7 +2676,7 @@
         <v>261</v>
       </c>
       <c r="D53" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -2684,7 +2690,7 @@
         <v>261</v>
       </c>
       <c r="D54" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -2698,7 +2704,7 @@
         <v>261</v>
       </c>
       <c r="D55" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -2709,10 +2715,10 @@
         <v>259</v>
       </c>
       <c r="C56" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="D56" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -2726,7 +2732,7 @@
         <v>259</v>
       </c>
       <c r="D57" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -2740,7 +2746,7 @@
         <v>259</v>
       </c>
       <c r="D58" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -2754,7 +2760,7 @@
         <v>261</v>
       </c>
       <c r="D59" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -2768,7 +2774,7 @@
         <v>259</v>
       </c>
       <c r="D60" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -2782,7 +2788,7 @@
         <v>259</v>
       </c>
       <c r="D61" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -2793,10 +2799,10 @@
         <v>259</v>
       </c>
       <c r="C62" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D62" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -2810,7 +2816,7 @@
         <v>263</v>
       </c>
       <c r="D63" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -2824,7 +2830,7 @@
         <v>261</v>
       </c>
       <c r="D64" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -2838,7 +2844,7 @@
         <v>261</v>
       </c>
       <c r="D65" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -2852,7 +2858,7 @@
         <v>263</v>
       </c>
       <c r="D66" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -2866,7 +2872,7 @@
         <v>261</v>
       </c>
       <c r="D67" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -2880,7 +2886,7 @@
         <v>262</v>
       </c>
       <c r="D68" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -2894,7 +2900,7 @@
         <v>262</v>
       </c>
       <c r="D69" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -2908,7 +2914,7 @@
         <v>261</v>
       </c>
       <c r="D70" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -2922,7 +2928,7 @@
         <v>262</v>
       </c>
       <c r="D71" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -2936,7 +2942,7 @@
         <v>261</v>
       </c>
       <c r="D72" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -2950,7 +2956,7 @@
         <v>263</v>
       </c>
       <c r="D73" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -2964,7 +2970,7 @@
         <v>263</v>
       </c>
       <c r="D74" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -2978,7 +2984,7 @@
         <v>263</v>
       </c>
       <c r="D75" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -2992,7 +2998,7 @@
         <v>263</v>
       </c>
       <c r="D76" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -3006,7 +3012,7 @@
         <v>259</v>
       </c>
       <c r="D77" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -3020,7 +3026,7 @@
         <v>260</v>
       </c>
       <c r="D78" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -3034,7 +3040,7 @@
         <v>260</v>
       </c>
       <c r="D79" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -3045,10 +3051,10 @@
         <v>260</v>
       </c>
       <c r="C80" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D80" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -3059,10 +3065,10 @@
         <v>260</v>
       </c>
       <c r="C81" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D81" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -3076,7 +3082,7 @@
         <v>260</v>
       </c>
       <c r="D82" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -3090,7 +3096,7 @@
         <v>263</v>
       </c>
       <c r="D83" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -3104,7 +3110,7 @@
         <v>263</v>
       </c>
       <c r="D84" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -3118,7 +3124,7 @@
         <v>263</v>
       </c>
       <c r="D85" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -3132,7 +3138,7 @@
         <v>263</v>
       </c>
       <c r="D86" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -3146,7 +3152,7 @@
         <v>263</v>
       </c>
       <c r="D87" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -3160,7 +3166,7 @@
         <v>263</v>
       </c>
       <c r="D88" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -3174,7 +3180,7 @@
         <v>259</v>
       </c>
       <c r="D89" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -3188,7 +3194,7 @@
         <v>259</v>
       </c>
       <c r="D90" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -3202,7 +3208,7 @@
         <v>259</v>
       </c>
       <c r="D91" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -3216,7 +3222,7 @@
         <v>259</v>
       </c>
       <c r="D92" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -3230,7 +3236,7 @@
         <v>259</v>
       </c>
       <c r="D93" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -3244,7 +3250,7 @@
         <v>259</v>
       </c>
       <c r="D94" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -3258,7 +3264,7 @@
         <v>259</v>
       </c>
       <c r="D95" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -3272,7 +3278,7 @@
         <v>259</v>
       </c>
       <c r="D96" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -3286,7 +3292,7 @@
         <v>259</v>
       </c>
       <c r="D97" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
     </row>
     <row r="98" spans="1:4">
@@ -3300,7 +3306,7 @@
         <v>259</v>
       </c>
       <c r="D98" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -3314,7 +3320,7 @@
         <v>259</v>
       </c>
       <c r="D99" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="100" spans="1:4">
@@ -3328,7 +3334,7 @@
         <v>259</v>
       </c>
       <c r="D100" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="101" spans="1:4">
@@ -3342,7 +3348,7 @@
         <v>259</v>
       </c>
       <c r="D101" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -3356,7 +3362,7 @@
         <v>259</v>
       </c>
       <c r="D102" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
     <row r="103" spans="1:4">
@@ -3370,7 +3376,7 @@
         <v>259</v>
       </c>
       <c r="D103" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="104" spans="1:4">
@@ -3384,7 +3390,7 @@
         <v>259</v>
       </c>
       <c r="D104" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="105" spans="1:4">
@@ -3398,7 +3404,7 @@
         <v>261</v>
       </c>
       <c r="D105" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="106" spans="1:4">
@@ -3412,7 +3418,7 @@
         <v>261</v>
       </c>
       <c r="D106" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="107" spans="1:4">
@@ -3423,10 +3429,10 @@
         <v>259</v>
       </c>
       <c r="C107" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D107" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="108" spans="1:4">
@@ -3440,7 +3446,7 @@
         <v>261</v>
       </c>
       <c r="D108" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="109" spans="1:4">
@@ -3454,7 +3460,7 @@
         <v>262</v>
       </c>
       <c r="D109" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
     </row>
     <row r="110" spans="1:4">
@@ -3468,7 +3474,7 @@
         <v>262</v>
       </c>
       <c r="D110" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="111" spans="1:4">
@@ -3482,7 +3488,7 @@
         <v>262</v>
       </c>
       <c r="D111" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="112" spans="1:4">
@@ -3496,7 +3502,7 @@
         <v>262</v>
       </c>
       <c r="D112" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="113" spans="1:4">
@@ -3510,7 +3516,7 @@
         <v>262</v>
       </c>
       <c r="D113" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="114" spans="1:4">
@@ -3524,7 +3530,7 @@
         <v>262</v>
       </c>
       <c r="D114" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="115" spans="1:4">
@@ -3538,7 +3544,7 @@
         <v>262</v>
       </c>
       <c r="D115" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="116" spans="1:4">
@@ -3552,7 +3558,7 @@
         <v>261</v>
       </c>
       <c r="D116" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="117" spans="1:4">
@@ -3566,7 +3572,7 @@
         <v>261</v>
       </c>
       <c r="D117" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="118" spans="1:4">
@@ -3577,10 +3583,10 @@
         <v>259</v>
       </c>
       <c r="C118" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D118" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="119" spans="1:4">
@@ -3594,7 +3600,7 @@
         <v>261</v>
       </c>
       <c r="D119" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="120" spans="1:4">
@@ -3605,10 +3611,10 @@
         <v>262</v>
       </c>
       <c r="C120" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D120" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="121" spans="1:4">
@@ -3622,7 +3628,7 @@
         <v>262</v>
       </c>
       <c r="D121" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="122" spans="1:4">
@@ -3636,7 +3642,7 @@
         <v>262</v>
       </c>
       <c r="D122" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
     </row>
     <row r="123" spans="1:4">
@@ -3650,7 +3656,7 @@
         <v>262</v>
       </c>
       <c r="D123" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="124" spans="1:4">
@@ -3664,7 +3670,7 @@
         <v>263</v>
       </c>
       <c r="D124" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="125" spans="1:4">
@@ -3678,7 +3684,7 @@
         <v>262</v>
       </c>
       <c r="D125" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
     </row>
     <row r="126" spans="1:4">
@@ -3692,7 +3698,7 @@
         <v>262</v>
       </c>
       <c r="D126" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="127" spans="1:4">
@@ -3706,7 +3712,7 @@
         <v>262</v>
       </c>
       <c r="D127" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="128" spans="1:4">
@@ -3717,10 +3723,10 @@
         <v>259</v>
       </c>
       <c r="C128" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D128" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="129" spans="1:4">
@@ -3734,7 +3740,7 @@
         <v>259</v>
       </c>
       <c r="D129" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="130" spans="1:4">
@@ -3748,7 +3754,7 @@
         <v>259</v>
       </c>
       <c r="D130" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="131" spans="1:4">
@@ -3762,7 +3768,7 @@
         <v>259</v>
       </c>
       <c r="D131" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="132" spans="1:4">
@@ -3776,7 +3782,7 @@
         <v>259</v>
       </c>
       <c r="D132" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="133" spans="1:4">
@@ -3790,7 +3796,7 @@
         <v>262</v>
       </c>
       <c r="D133" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="134" spans="1:4">
@@ -3804,7 +3810,7 @@
         <v>259</v>
       </c>
       <c r="D134" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="135" spans="1:4">
@@ -3818,7 +3824,7 @@
         <v>259</v>
       </c>
       <c r="D135" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
     <row r="136" spans="1:4">
@@ -3832,7 +3838,7 @@
         <v>263</v>
       </c>
       <c r="D136" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
     </row>
     <row r="137" spans="1:4">
@@ -3846,7 +3852,7 @@
         <v>263</v>
       </c>
       <c r="D137" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="138" spans="1:4">
@@ -3860,7 +3866,7 @@
         <v>261</v>
       </c>
       <c r="D138" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="139" spans="1:4">
@@ -3874,7 +3880,7 @@
         <v>261</v>
       </c>
       <c r="D139" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="140" spans="1:4">
@@ -3888,7 +3894,7 @@
         <v>259</v>
       </c>
       <c r="D140" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
     </row>
     <row r="141" spans="1:4">
@@ -3899,10 +3905,10 @@
         <v>259</v>
       </c>
       <c r="C141" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D141" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
     </row>
     <row r="142" spans="1:4">
@@ -3916,7 +3922,7 @@
         <v>261</v>
       </c>
       <c r="D142" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="143" spans="1:4">
@@ -3930,7 +3936,7 @@
         <v>262</v>
       </c>
       <c r="D143" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="144" spans="1:4">
@@ -3944,7 +3950,7 @@
         <v>259</v>
       </c>
       <c r="D144" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
     <row r="145" spans="1:4">
@@ -3958,7 +3964,7 @@
         <v>260</v>
       </c>
       <c r="D145" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="146" spans="1:4">
@@ -3972,7 +3978,7 @@
         <v>260</v>
       </c>
       <c r="D146" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
     </row>
     <row r="147" spans="1:4">
@@ -3986,7 +3992,7 @@
         <v>259</v>
       </c>
       <c r="D147" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
     </row>
     <row r="148" spans="1:4">
@@ -4000,7 +4006,7 @@
         <v>263</v>
       </c>
       <c r="D148" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="149" spans="1:4">
@@ -4014,7 +4020,7 @@
         <v>259</v>
       </c>
       <c r="D149" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
     </row>
     <row r="150" spans="1:4">
@@ -4028,7 +4034,7 @@
         <v>262</v>
       </c>
       <c r="D150" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="151" spans="1:4">
@@ -4042,7 +4048,7 @@
         <v>259</v>
       </c>
       <c r="D151" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
     </row>
     <row r="152" spans="1:4">
@@ -4056,7 +4062,7 @@
         <v>262</v>
       </c>
       <c r="D152" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="153" spans="1:4">
@@ -4067,10 +4073,10 @@
         <v>259</v>
       </c>
       <c r="C153" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="D153" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
     </row>
     <row r="154" spans="1:4">
@@ -4084,7 +4090,7 @@
         <v>259</v>
       </c>
       <c r="D154" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
     </row>
     <row r="155" spans="1:4">
@@ -4098,7 +4104,7 @@
         <v>259</v>
       </c>
       <c r="D155" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
     </row>
     <row r="156" spans="1:4">
@@ -4112,7 +4118,7 @@
         <v>261</v>
       </c>
       <c r="D156" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="157" spans="1:4">
@@ -4126,7 +4132,7 @@
         <v>259</v>
       </c>
       <c r="D157" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
     </row>
     <row r="158" spans="1:4">
@@ -4140,7 +4146,7 @@
         <v>259</v>
       </c>
       <c r="D158" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
     </row>
     <row r="159" spans="1:4">
@@ -4154,7 +4160,7 @@
         <v>262</v>
       </c>
       <c r="D159" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
     </row>
     <row r="160" spans="1:4">
@@ -4165,10 +4171,10 @@
         <v>259</v>
       </c>
       <c r="C160" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D160" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
     </row>
     <row r="161" spans="1:4">
@@ -4182,7 +4188,7 @@
         <v>262</v>
       </c>
       <c r="D161" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
     </row>
     <row r="162" spans="1:4">
@@ -4196,7 +4202,7 @@
         <v>262</v>
       </c>
       <c r="D162" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="163" spans="1:4">
@@ -4210,7 +4216,7 @@
         <v>262</v>
       </c>
       <c r="D163" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
     </row>
     <row r="164" spans="1:4">
@@ -4224,7 +4230,7 @@
         <v>262</v>
       </c>
       <c r="D164" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
     </row>
     <row r="165" spans="1:4">
@@ -4238,7 +4244,7 @@
         <v>259</v>
       </c>
       <c r="D165" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="166" spans="1:4">
@@ -4252,7 +4258,7 @@
         <v>259</v>
       </c>
       <c r="D166" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="167" spans="1:4">
@@ -4266,7 +4272,7 @@
         <v>259</v>
       </c>
       <c r="D167" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="168" spans="1:4">
@@ -4280,7 +4286,7 @@
         <v>259</v>
       </c>
       <c r="D168" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="169" spans="1:4">
@@ -4294,7 +4300,7 @@
         <v>259</v>
       </c>
       <c r="D169" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="170" spans="1:4">
@@ -4308,7 +4314,7 @@
         <v>259</v>
       </c>
       <c r="D170" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
     <row r="171" spans="1:4">
@@ -4322,7 +4328,7 @@
         <v>259</v>
       </c>
       <c r="D171" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="172" spans="1:4">
@@ -4336,7 +4342,7 @@
         <v>259</v>
       </c>
       <c r="D172" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
     </row>
     <row r="173" spans="1:4">
@@ -4350,7 +4356,7 @@
         <v>262</v>
       </c>
       <c r="D173" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="174" spans="1:4">
@@ -4364,7 +4370,7 @@
         <v>262</v>
       </c>
       <c r="D174" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
     </row>
     <row r="175" spans="1:4">
@@ -4378,7 +4384,7 @@
         <v>262</v>
       </c>
       <c r="D175" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="176" spans="1:4">
@@ -4389,10 +4395,10 @@
         <v>261</v>
       </c>
       <c r="C176" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D176" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="177" spans="1:4">
@@ -4406,7 +4412,7 @@
         <v>262</v>
       </c>
       <c r="D177" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="178" spans="1:4">
@@ -4417,10 +4423,10 @@
         <v>259</v>
       </c>
       <c r="C178" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D178" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
     </row>
     <row r="179" spans="1:4">
@@ -4434,7 +4440,7 @@
         <v>262</v>
       </c>
       <c r="D179" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="180" spans="1:4">
@@ -4448,7 +4454,7 @@
         <v>262</v>
       </c>
       <c r="D180" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="181" spans="1:4">
@@ -4462,7 +4468,7 @@
         <v>261</v>
       </c>
       <c r="D181" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
     <row r="182" spans="1:4">
@@ -4473,10 +4479,10 @@
         <v>259</v>
       </c>
       <c r="C182" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="D182" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
     </row>
     <row r="183" spans="1:4">
@@ -4490,7 +4496,7 @@
         <v>261</v>
       </c>
       <c r="D183" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
     </row>
     <row r="184" spans="1:4">
@@ -4504,7 +4510,7 @@
         <v>261</v>
       </c>
       <c r="D184" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
     </row>
     <row r="185" spans="1:4">
@@ -4518,7 +4524,7 @@
         <v>261</v>
       </c>
       <c r="D185" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
     </row>
     <row r="186" spans="1:4">
@@ -4532,7 +4538,7 @@
         <v>261</v>
       </c>
       <c r="D186" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
     </row>
     <row r="187" spans="1:4">
@@ -4546,7 +4552,7 @@
         <v>261</v>
       </c>
       <c r="D187" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
     </row>
     <row r="188" spans="1:4">
@@ -4560,7 +4566,7 @@
         <v>261</v>
       </c>
       <c r="D188" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
     </row>
     <row r="189" spans="1:4">
@@ -4574,7 +4580,7 @@
         <v>261</v>
       </c>
       <c r="D189" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
     </row>
     <row r="190" spans="1:4">
@@ -4588,7 +4594,7 @@
         <v>261</v>
       </c>
       <c r="D190" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
     </row>
     <row r="191" spans="1:4">
@@ -4599,10 +4605,10 @@
         <v>259</v>
       </c>
       <c r="C191" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D191" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
     </row>
     <row r="192" spans="1:4">
@@ -4613,10 +4619,10 @@
         <v>259</v>
       </c>
       <c r="C192" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D192" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
     </row>
     <row r="193" spans="1:4">
@@ -4630,7 +4636,7 @@
         <v>261</v>
       </c>
       <c r="D193" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
     </row>
     <row r="194" spans="1:4">
@@ -4641,10 +4647,10 @@
         <v>261</v>
       </c>
       <c r="C194" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D194" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
     </row>
     <row r="195" spans="1:4">
@@ -4655,10 +4661,10 @@
         <v>261</v>
       </c>
       <c r="C195" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D195" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
     </row>
     <row r="196" spans="1:4">
@@ -4669,10 +4675,10 @@
         <v>259</v>
       </c>
       <c r="C196" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D196" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
     </row>
     <row r="197" spans="1:4">
@@ -4686,7 +4692,7 @@
         <v>262</v>
       </c>
       <c r="D197" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
     </row>
     <row r="198" spans="1:4">
@@ -4700,7 +4706,7 @@
         <v>262</v>
       </c>
       <c r="D198" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
     </row>
     <row r="199" spans="1:4">
@@ -4714,7 +4720,7 @@
         <v>262</v>
       </c>
       <c r="D199" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="200" spans="1:4">
@@ -4728,7 +4734,7 @@
         <v>262</v>
       </c>
       <c r="D200" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
     </row>
     <row r="201" spans="1:4">
@@ -4742,7 +4748,7 @@
         <v>262</v>
       </c>
       <c r="D201" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="202" spans="1:4">
@@ -4756,7 +4762,7 @@
         <v>262</v>
       </c>
       <c r="D202" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
     </row>
     <row r="203" spans="1:4">
@@ -4770,7 +4776,7 @@
         <v>262</v>
       </c>
       <c r="D203" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
     </row>
     <row r="204" spans="1:4">
@@ -4781,10 +4787,10 @@
         <v>259</v>
       </c>
       <c r="C204" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D204" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
     </row>
     <row r="205" spans="1:4">
@@ -4798,7 +4804,7 @@
         <v>259</v>
       </c>
       <c r="D205" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
     </row>
     <row r="206" spans="1:4">
@@ -4812,7 +4818,7 @@
         <v>261</v>
       </c>
       <c r="D206" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
     </row>
     <row r="207" spans="1:4">
@@ -4826,7 +4832,7 @@
         <v>261</v>
       </c>
       <c r="D207" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
     </row>
     <row r="208" spans="1:4">
@@ -4840,7 +4846,7 @@
         <v>261</v>
       </c>
       <c r="D208" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
     </row>
     <row r="209" spans="1:4">
@@ -4854,7 +4860,7 @@
         <v>261</v>
       </c>
       <c r="D209" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="210" spans="1:4">
@@ -4868,7 +4874,7 @@
         <v>261</v>
       </c>
       <c r="D210" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="211" spans="1:4">
@@ -4882,7 +4888,7 @@
         <v>261</v>
       </c>
       <c r="D211" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
     </row>
     <row r="212" spans="1:4">
@@ -4893,10 +4899,10 @@
         <v>261</v>
       </c>
       <c r="C212" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D212" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
     </row>
     <row r="213" spans="1:4">
@@ -4910,7 +4916,7 @@
         <v>259</v>
       </c>
       <c r="D213" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
     <row r="214" spans="1:4">
@@ -4924,7 +4930,7 @@
         <v>259</v>
       </c>
       <c r="D214" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
     </row>
     <row r="215" spans="1:4">
@@ -4938,7 +4944,7 @@
         <v>259</v>
       </c>
       <c r="D215" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
     </row>
     <row r="216" spans="1:4">
@@ -4952,7 +4958,7 @@
         <v>259</v>
       </c>
       <c r="D216" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
     </row>
     <row r="217" spans="1:4">
@@ -4966,7 +4972,7 @@
         <v>259</v>
       </c>
       <c r="D217" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
     </row>
     <row r="218" spans="1:4">
@@ -4980,7 +4986,7 @@
         <v>259</v>
       </c>
       <c r="D218" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="219" spans="1:4">
@@ -4994,7 +5000,7 @@
         <v>259</v>
       </c>
       <c r="D219" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="220" spans="1:4">
@@ -5008,7 +5014,7 @@
         <v>259</v>
       </c>
       <c r="D220" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="221" spans="1:4">
@@ -5022,7 +5028,7 @@
         <v>261</v>
       </c>
       <c r="D221" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="222" spans="1:4">
@@ -5036,7 +5042,7 @@
         <v>262</v>
       </c>
       <c r="D222" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="223" spans="1:4">
@@ -5050,7 +5056,7 @@
         <v>259</v>
       </c>
       <c r="D223" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="224" spans="1:4">
@@ -5064,7 +5070,7 @@
         <v>261</v>
       </c>
       <c r="D224" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="225" spans="1:4">
@@ -5078,7 +5084,7 @@
         <v>261</v>
       </c>
       <c r="D225" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="226" spans="1:4">
@@ -5092,7 +5098,7 @@
         <v>261</v>
       </c>
       <c r="D226" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -5106,7 +5112,7 @@
         <v>261</v>
       </c>
       <c r="D227" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="228" spans="1:4">
@@ -5120,7 +5126,7 @@
         <v>261</v>
       </c>
       <c r="D228" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -5134,7 +5140,7 @@
         <v>261</v>
       </c>
       <c r="D229" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="230" spans="1:4">
@@ -5148,7 +5154,7 @@
         <v>261</v>
       </c>
       <c r="D230" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="231" spans="1:4">
@@ -5162,7 +5168,7 @@
         <v>261</v>
       </c>
       <c r="D231" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="232" spans="1:4">
@@ -5173,10 +5179,10 @@
         <v>259</v>
       </c>
       <c r="C232" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D232" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="233" spans="1:4">
@@ -5187,10 +5193,10 @@
         <v>259</v>
       </c>
       <c r="C233" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D233" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="234" spans="1:4">
@@ -5201,10 +5207,10 @@
         <v>259</v>
       </c>
       <c r="C234" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D234" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="235" spans="1:4">
@@ -5218,7 +5224,7 @@
         <v>259</v>
       </c>
       <c r="D235" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="236" spans="1:4">
@@ -5232,7 +5238,7 @@
         <v>259</v>
       </c>
       <c r="D236" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="237" spans="1:4">
@@ -5246,7 +5252,7 @@
         <v>259</v>
       </c>
       <c r="D237" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="238" spans="1:4">
@@ -5260,7 +5266,7 @@
         <v>259</v>
       </c>
       <c r="D238" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="239" spans="1:4">
@@ -5274,7 +5280,7 @@
         <v>259</v>
       </c>
       <c r="D239" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="240" spans="1:4">
@@ -5288,7 +5294,7 @@
         <v>259</v>
       </c>
       <c r="D240" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="241" spans="1:4">
@@ -5302,7 +5308,7 @@
         <v>259</v>
       </c>
       <c r="D241" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="242" spans="1:4">
@@ -5316,7 +5322,7 @@
         <v>259</v>
       </c>
       <c r="D242" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="243" spans="1:4">
@@ -5330,7 +5336,7 @@
         <v>261</v>
       </c>
       <c r="D243" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="244" spans="1:4">
@@ -5344,7 +5350,7 @@
         <v>261</v>
       </c>
       <c r="D244" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="245" spans="1:4">
@@ -5358,7 +5364,7 @@
         <v>261</v>
       </c>
       <c r="D245" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="246" spans="1:4">
@@ -5369,10 +5375,10 @@
         <v>261</v>
       </c>
       <c r="C246" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D246" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="247" spans="1:4">
@@ -5386,7 +5392,7 @@
         <v>261</v>
       </c>
       <c r="D247" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="248" spans="1:4">
@@ -5400,7 +5406,7 @@
         <v>261</v>
       </c>
       <c r="D248" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="249" spans="1:4">
@@ -5414,7 +5420,7 @@
         <v>261</v>
       </c>
       <c r="D249" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="250" spans="1:4">
@@ -5428,7 +5434,7 @@
         <v>261</v>
       </c>
       <c r="D250" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="251" spans="1:4">
@@ -5442,7 +5448,7 @@
         <v>259</v>
       </c>
       <c r="D251" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="252" spans="1:4">
@@ -5456,7 +5462,7 @@
         <v>259</v>
       </c>
       <c r="D252" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="253" spans="1:4">
@@ -5470,7 +5476,7 @@
         <v>259</v>
       </c>
       <c r="D253" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
     </row>
     <row r="254" spans="1:4">
@@ -5484,7 +5490,7 @@
         <v>260</v>
       </c>
       <c r="D254" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
     </row>
     <row r="255" spans="1:4">
@@ -5498,7 +5504,7 @@
         <v>260</v>
       </c>
       <c r="D255" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="256" spans="1:4">
@@ -5512,7 +5518,7 @@
         <v>262</v>
       </c>
       <c r="D256" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
     </row>
   </sheetData>

</xml_diff>